<commit_message>
Pendent de posar la finestra en una pestanya.
--HG--
branch : Desgloç Per IRPF
</commit_message>
<xml_diff>
--- a/Docs/Desglo� per IRPF.xlsx
+++ b/Docs/Desglo� per IRPF.xlsx
@@ -8,10 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C06CAE-5C9D-400A-A03B-121292D5C516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AC34FF-3CD9-48C6-A569-53166343FB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{D5391FB0-AD89-473B-AA62-C3B5FCAECA9A}"/>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{C13071D3-7DC4-40C4-95BF-6C65EC911B05}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{D5391FB0-AD89-473B-AA62-C3B5FCAECA9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hisenda" sheetId="1" r:id="rId1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
   <si>
     <t>PiG ---&gt;</t>
   </si>
@@ -144,6 +143,15 @@
   </si>
   <si>
     <t>Participacions utilitzades</t>
+  </si>
+  <si>
+    <t>Desp C</t>
+  </si>
+  <si>
+    <t>Desp V</t>
+  </si>
+  <si>
+    <t>Desp Ut</t>
   </si>
 </sst>
 </file>
@@ -493,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -682,6 +690,8 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -996,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{386CFA17-404F-4DA8-8891-F2A744C8D48D}">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
@@ -1238,6 +1248,10 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
+      <c r="A9" s="62"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
       <c r="F9" s="76">
         <v>44559</v>
       </c>
@@ -1258,7 +1272,17 @@
         <v>-900</v>
       </c>
     </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="62"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+    </row>
     <row r="11" spans="1:11">
+      <c r="A11" s="62"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
       <c r="F11" s="81" t="s">
         <v>28</v>
       </c>
@@ -1267,10 +1291,38 @@
       <c r="I11" s="81"/>
     </row>
     <row r="12" spans="1:11">
+      <c r="A12" s="62"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
       <c r="F12" s="82" t="s">
         <v>35</v>
       </c>
       <c r="G12" s="82"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="62"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="D14" s="62"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="D15" s="62"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="D16" s="62"/>
+    </row>
+    <row r="17" spans="4:4">
+      <c r="D17" s="62"/>
+    </row>
+    <row r="18" spans="4:4">
+      <c r="D18" s="62"/>
+    </row>
+    <row r="19" spans="4:4">
+      <c r="D19" s="62"/>
+    </row>
+    <row r="20" spans="4:4">
+      <c r="D20" s="85"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1280,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5D9BEC9-2BA1-4AC7-AE63-E9CBF2F6D6B4}">
-  <dimension ref="B1:P28"/>
+  <dimension ref="B1:S28"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -1294,11 +1346,10 @@
     <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="1.26953125" customWidth="1"/>
     <col min="13" max="14" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="3.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16">
+    <row r="1" spans="2:19">
       <c r="D1" s="12" t="s">
         <v>4</v>
       </c>
@@ -1319,7 +1370,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="2:16">
+    <row r="2" spans="2:19">
       <c r="B2" s="3">
         <v>166</v>
       </c>
@@ -1353,7 +1404,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="3" spans="2:16">
+    <row r="3" spans="2:19">
       <c r="B3" s="3">
         <v>169</v>
       </c>
@@ -1387,7 +1438,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="4" spans="2:16">
+    <row r="4" spans="2:19">
       <c r="B4" s="3">
         <v>174</v>
       </c>
@@ -1421,7 +1472,7 @@
         <v>1652</v>
       </c>
     </row>
-    <row r="5" spans="2:16">
+    <row r="5" spans="2:19">
       <c r="B5" s="6">
         <v>176</v>
       </c>
@@ -1455,7 +1506,7 @@
         <v>1652</v>
       </c>
     </row>
-    <row r="6" spans="2:16">
+    <row r="6" spans="2:19">
       <c r="B6" s="3">
         <v>177</v>
       </c>
@@ -1489,7 +1540,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="2:16">
+    <row r="7" spans="2:19">
       <c r="B7" s="3">
         <v>178</v>
       </c>
@@ -1525,8 +1576,17 @@
       <c r="M7" s="44">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="2:16">
+      <c r="Q7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R7" t="s">
+        <v>37</v>
+      </c>
+      <c r="S7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19">
       <c r="B8" s="3">
         <v>191</v>
       </c>
@@ -1570,9 +1630,24 @@
         <f>E8-M8-N8</f>
         <v>254</v>
       </c>
-      <c r="P8" s="9"/>
-    </row>
-    <row r="9" spans="2:16">
+      <c r="P8" s="9">
+        <f>SUM(N8:O8)</f>
+        <v>308</v>
+      </c>
+      <c r="Q8" s="62">
+        <f>J8/E8*P8</f>
+        <v>4.7459999999999996</v>
+      </c>
+      <c r="R8" s="62">
+        <f>J15+J16/E16*O8</f>
+        <v>3.4802600472813237</v>
+      </c>
+      <c r="S8" s="62">
+        <f>+Q8+R8</f>
+        <v>8.2262600472813237</v>
+      </c>
+    </row>
+    <row r="9" spans="2:19">
       <c r="B9" s="3">
         <v>190</v>
       </c>
@@ -1609,8 +1684,24 @@
         <f>E9</f>
         <v>92</v>
       </c>
-    </row>
-    <row r="10" spans="2:16">
+      <c r="P9" s="9">
+        <f>SUM(M9:O9)</f>
+        <v>92</v>
+      </c>
+      <c r="Q9" s="62">
+        <f>J9</f>
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="R9" s="62">
+        <f>J$16/E$16*M9</f>
+        <v>1.0396217494089834</v>
+      </c>
+      <c r="S9" s="62">
+        <f t="shared" ref="S9:S12" si="2">+Q9+R9</f>
+        <v>6.0996217494089828</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19">
       <c r="B10" s="3">
         <v>179</v>
       </c>
@@ -1643,8 +1734,9 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-    </row>
-    <row r="11" spans="2:16">
+      <c r="S10" s="62"/>
+    </row>
+    <row r="11" spans="2:19">
       <c r="B11" s="3">
         <v>193</v>
       </c>
@@ -1681,8 +1773,24 @@
         <f>E11</f>
         <v>433</v>
       </c>
-    </row>
-    <row r="12" spans="2:16">
+      <c r="P11" s="9">
+        <f>SUM(M11:O11)</f>
+        <v>433</v>
+      </c>
+      <c r="Q11" s="62">
+        <f>J11</f>
+        <v>8.06</v>
+      </c>
+      <c r="R11" s="62">
+        <f>J$16/E$16*M11</f>
+        <v>4.8930023640661942</v>
+      </c>
+      <c r="S11" s="62">
+        <f t="shared" si="2"/>
+        <v>12.953002364066194</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19">
       <c r="B12" s="3">
         <v>192</v>
       </c>
@@ -1719,8 +1827,24 @@
         <f>E16-O8-M9-M11</f>
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="2:16" ht="15" thickBot="1">
+      <c r="P12" s="9">
+        <f>SUM(M12:O12)</f>
+        <v>67</v>
+      </c>
+      <c r="Q12" s="62">
+        <f>J12/E12*P12</f>
+        <v>1.3480400000000001</v>
+      </c>
+      <c r="R12" s="62">
+        <f>J$16/E$16*M12</f>
+        <v>0.75711583924349879</v>
+      </c>
+      <c r="S12" s="62">
+        <f t="shared" si="2"/>
+        <v>2.105155839243499</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" ht="15" thickBot="1">
       <c r="B13" s="3">
         <v>182</v>
       </c>
@@ -1755,7 +1879,7 @@
       </c>
       <c r="M13" s="9"/>
     </row>
-    <row r="14" spans="2:16">
+    <row r="14" spans="2:19">
       <c r="B14" s="6">
         <v>195</v>
       </c>
@@ -1795,7 +1919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:16">
+    <row r="15" spans="2:19">
       <c r="B15" s="3">
         <v>206</v>
       </c>
@@ -1836,8 +1960,12 @@
         <f>G15</f>
         <v>1544.4</v>
       </c>
-    </row>
-    <row r="16" spans="2:16" ht="15" thickBot="1">
+      <c r="Q15" s="62">
+        <f>J15</f>
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" ht="15" thickBot="1">
       <c r="B16" s="3">
         <v>207</v>
       </c>
@@ -1878,8 +2006,12 @@
         <f>G16</f>
         <v>24195.599999999999</v>
       </c>
-    </row>
-    <row r="17" spans="2:14" ht="15" thickBot="1">
+      <c r="Q16" s="62">
+        <f>J16</f>
+        <v>9.56</v>
+      </c>
+    </row>
+    <row r="17" spans="2:17" ht="15" thickBot="1">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="4"/>
@@ -1899,8 +2031,12 @@
         <f>SUM(N15:N16)</f>
         <v>25740</v>
       </c>
-    </row>
-    <row r="18" spans="2:14">
+      <c r="Q17" s="84">
+        <f>SUM(Q8:Q16)</f>
+        <v>29.384039999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:17">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="4"/>
@@ -1920,7 +2056,7 @@
         <v>12970.75</v>
       </c>
     </row>
-    <row r="19" spans="2:14">
+    <row r="19" spans="2:17">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="4"/>
@@ -1940,7 +2076,7 @@
         <v>29.384039999999999</v>
       </c>
     </row>
-    <row r="20" spans="2:14">
+    <row r="20" spans="2:17">
       <c r="B20" s="3">
         <v>208</v>
       </c>
@@ -1964,7 +2100,7 @@
         <v>12941.365959999999</v>
       </c>
     </row>
-    <row r="21" spans="2:14">
+    <row r="21" spans="2:17">
       <c r="B21" s="3">
         <v>209</v>
       </c>
@@ -1988,7 +2124,7 @@
         <v>12941.689999999997</v>
       </c>
     </row>
-    <row r="22" spans="2:14" ht="15" thickBot="1">
+    <row r="22" spans="2:17" ht="15" thickBot="1">
       <c r="B22" s="3">
         <v>210</v>
       </c>
@@ -2012,7 +2148,7 @@
         <v>-0.32403999999769439</v>
       </c>
     </row>
-    <row r="23" spans="2:14">
+    <row r="23" spans="2:17">
       <c r="B23" s="3">
         <v>211</v>
       </c>
@@ -2029,7 +2165,7 @@
       <c r="K23" s="3"/>
       <c r="L23" s="9"/>
     </row>
-    <row r="24" spans="2:14">
+    <row r="24" spans="2:17">
       <c r="B24" s="3">
         <v>212</v>
       </c>
@@ -2046,7 +2182,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="9"/>
     </row>
-    <row r="25" spans="2:14">
+    <row r="25" spans="2:17">
       <c r="B25" s="3">
         <v>213</v>
       </c>
@@ -2063,7 +2199,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="9"/>
     </row>
-    <row r="26" spans="2:14">
+    <row r="26" spans="2:17">
       <c r="B26" s="3">
         <v>214</v>
       </c>
@@ -2080,7 +2216,7 @@
       <c r="K26" s="3"/>
       <c r="L26" s="9"/>
     </row>
-    <row r="27" spans="2:14">
+    <row r="27" spans="2:17">
       <c r="B27" s="3">
         <v>215</v>
       </c>
@@ -2097,11 +2233,12 @@
       <c r="K27" s="3"/>
       <c r="L27" s="9"/>
     </row>
-    <row r="28" spans="2:14">
+    <row r="28" spans="2:17">
       <c r="E28" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="N21" formula="1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Reanonat de particions a participacions.
</commit_message>
<xml_diff>
--- a/Docs/Desglo� per IRPF.xlsx
+++ b/Docs/Desglo� per IRPF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AC34FF-3CD9-48C6-A569-53166343FB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB9BE59-CE3A-405D-8384-0EC5B15C90BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{D5391FB0-AD89-473B-AA62-C3B5FCAECA9A}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5391FB0-AD89-473B-AA62-C3B5FCAECA9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hisenda" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="40">
   <si>
     <t>PiG ---&gt;</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Desp Ut</t>
+  </si>
+  <si>
+    <t>Perdues anys anterios</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1012,8 @@
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="2" customWidth="1"/>
     <col min="6" max="6" width="8.08984375" bestFit="1" customWidth="1"/>
@@ -1248,7 +1252,9 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
-      <c r="A9" s="62"/>
+      <c r="A9" s="84" t="s">
+        <v>39</v>
+      </c>
       <c r="B9" s="62"/>
       <c r="C9" s="62"/>
       <c r="D9" s="62"/>
@@ -1273,7 +1279,9 @@
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="62"/>
+      <c r="A10" s="84">
+        <v>5845.75</v>
+      </c>
       <c r="B10" s="62"/>
       <c r="C10" s="62"/>
       <c r="D10" s="62"/>

</xml_diff>